<commit_message>
BOM fixes: 342mm X extrusion, MGN9H typo, Front Left plate names
Spreadsheet corrections; BOM.md regenerated from it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Printed Version/SV08_P6_Printed_BOM_from_STEP.xlsx
+++ b/Printed Version/SV08_P6_Printed_BOM_from_STEP.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8b9eab14d89956a8/3d Printing Stuff/Models/SV08 Mods/SV08 AWD Live Idlers Front Tensioners - Final/Printed Version/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="81" documentId="11_DFF688E9926BEE6F6450CCD7565DCE3A87C03B69" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C272D8FA-017C-496C-A6E1-24E1BA0760A1}"/>
+  <xr:revisionPtr revIDLastSave="89" documentId="11_DFF688E9926BEE6F6450CCD7565DCE3A87C03B69" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{36EC1B92-0323-4BDC-93AC-3015D06D29B3}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-51720" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Consolidated BOM" sheetId="1" r:id="rId1"/>
@@ -25,9 +25,6 @@
     <t>SV08-P6 Dual Shear Live Idlers Front Tensioners (Printed 6mm) — BOM (Extracted from STEP)</t>
   </si>
   <si>
-    <t>From the STEP tree. Z Carriages excluded, D2F-L switches counted as one unit each. Printed-plate version: all 12 plates are under Printed Parts. No open items. Hidden imported-model parts (e.g. the Xol carriage shim) are intentionally excluded. Purchase Links not merged (Drive file not pointed to this run).</t>
-  </si>
-  <si>
     <t>Category</t>
   </si>
   <si>
@@ -262,9 +259,6 @@
     <t>Linear Rails &amp; Sliders</t>
   </si>
   <si>
-    <t>MG9H Linear Rail Slide</t>
-  </si>
-  <si>
     <t>Y MGN9H Rail 402mm</t>
   </si>
   <si>
@@ -286,9 +280,6 @@
     <t>Gantry Y-Axis 2020 Extrusion 469mm</t>
   </si>
   <si>
-    <t>Gantry X-Axis 2020 Extrusion 357mm</t>
-  </si>
-  <si>
     <t>Shortened from 345mm: all tensioning now happens at the front motor mounts.</t>
   </si>
   <si>
@@ -331,12 +322,6 @@
     <t>Back Right Top Plate Printed6mm</t>
   </si>
   <si>
-    <t>Front Left Bottom Dual Shear Live Idler Tensioner Dual Lever</t>
-  </si>
-  <si>
-    <t>Front Left Top Dual Shear Live Idler Tensioner Dual Lever</t>
-  </si>
-  <si>
     <t>Front Right Bottom Printed6mm</t>
   </si>
   <si>
@@ -488,6 +473,21 @@
   </si>
   <si>
     <t>6mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions.</t>
+  </si>
+  <si>
+    <t>From the STEP tree. Z Carriages excluded, D2F-L switches counted as one unit each. Printed-plate version: all 12 plates are under Printed Parts. No open items. Hidden imported-model parts (e.g. the Xol carriage shim) are intentionally excluded.</t>
+  </si>
+  <si>
+    <t>Gantry X-Axis 2020 Extrusion 342mm</t>
+  </si>
+  <si>
+    <t>Front Left Bottom Printed6mm</t>
+  </si>
+  <si>
+    <t>Front Left Top Printed6mm</t>
+  </si>
+  <si>
+    <t>MGN9H Linear Rail Slide</t>
   </si>
 </sst>
 </file>
@@ -589,9 +589,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -610,6 +610,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -908,7 +912,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="6"/>
@@ -918,7 +922,7 @@
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="8" t="s">
-        <v>1</v>
+        <v>151</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -927,24 +931,24 @@
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="D4" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="E4" s="1" t="s">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="7" t="s">
         <v>5</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" s="5" t="s">
-        <v>6</v>
       </c>
       <c r="B5" s="6"/>
       <c r="C5" s="6"/>
@@ -953,161 +957,161 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B6" s="3">
         <v>28</v>
       </c>
       <c r="C6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>8</v>
-      </c>
-      <c r="D6" t="s">
-        <v>113</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B7" s="3">
         <v>28</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D7" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="E7" s="2"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B8" s="3">
         <v>24</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B9" s="3">
         <v>16</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D9" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="E9" s="2"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B10" s="3">
         <v>8</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D10" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11" s="3">
         <v>8</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D11" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="E11" s="2"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B12" s="3">
         <v>4</v>
       </c>
       <c r="C12" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" t="s">
+        <v>113</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="D12" t="s">
-        <v>118</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B13" s="3">
         <v>4</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D13" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="E13" s="2"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B14" s="3">
         <v>4</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D14" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="E14" s="2"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B15" s="3">
         <v>4</v>
       </c>
       <c r="C15" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" t="s">
+        <v>116</v>
+      </c>
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A16" s="7" t="s">
         <v>19</v>
-      </c>
-      <c r="D15" t="s">
-        <v>121</v>
-      </c>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>20</v>
       </c>
       <c r="B16" s="6"/>
       <c r="C16" s="6"/>
@@ -1116,58 +1120,58 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B17" s="3">
         <v>8</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D17" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18" s="3">
         <v>4</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D18" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B19" s="3">
         <v>4</v>
       </c>
       <c r="C19" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D19" t="s">
+        <v>139</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" s="7" t="s">
         <v>24</v>
-      </c>
-      <c r="D19" t="s">
-        <v>144</v>
-      </c>
-      <c r="E19" s="4" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="5" t="s">
-        <v>25</v>
       </c>
       <c r="B20" s="6"/>
       <c r="C20" s="6"/>
@@ -1176,37 +1180,37 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B21" s="3">
         <v>32</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D21" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="E21" s="2"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B22" s="3">
         <v>28</v>
       </c>
       <c r="C22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D22" t="s">
+        <v>118</v>
+      </c>
+      <c r="E22" s="2"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="7" t="s">
         <v>28</v>
-      </c>
-      <c r="D22" t="s">
-        <v>123</v>
-      </c>
-      <c r="E22" s="2"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="5" t="s">
-        <v>29</v>
       </c>
       <c r="B23" s="6"/>
       <c r="C23" s="6"/>
@@ -1215,24 +1219,24 @@
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B24" s="3">
         <v>2</v>
       </c>
       <c r="C24" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D24" t="s">
+        <v>119</v>
+      </c>
+      <c r="E24" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D24" t="s">
-        <v>124</v>
-      </c>
-      <c r="E24" s="4" t="s">
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
         <v>32</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="5" t="s">
-        <v>33</v>
       </c>
       <c r="B25" s="6"/>
       <c r="C25" s="6"/>
@@ -1241,24 +1245,24 @@
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B26" s="3">
         <v>2</v>
       </c>
       <c r="C26" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="D26" t="s">
+        <v>120</v>
+      </c>
+      <c r="E26" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D26" t="s">
-        <v>125</v>
-      </c>
-      <c r="E26" s="4" t="s">
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" s="7" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="5" t="s">
-        <v>37</v>
       </c>
       <c r="B27" s="6"/>
       <c r="C27" s="6"/>
@@ -1267,37 +1271,37 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B28" s="3">
         <v>4</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D28" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="E28" s="2"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B29" s="3">
         <v>4</v>
       </c>
       <c r="C29" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" t="s">
+        <v>122</v>
+      </c>
+      <c r="E29" s="2"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" s="7" t="s">
         <v>40</v>
-      </c>
-      <c r="D29" t="s">
-        <v>127</v>
-      </c>
-      <c r="E29" s="2"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="5" t="s">
-        <v>41</v>
       </c>
       <c r="B30" s="6"/>
       <c r="C30" s="6"/>
@@ -1306,24 +1310,24 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B31" s="3">
         <v>36</v>
       </c>
       <c r="C31" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D31" t="s">
+        <v>123</v>
+      </c>
+      <c r="E31" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D31" t="s">
-        <v>128</v>
-      </c>
-      <c r="E31" s="4" t="s">
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
         <v>44</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="5" t="s">
-        <v>45</v>
       </c>
       <c r="B32" s="6"/>
       <c r="C32" s="6"/>
@@ -1332,71 +1336,71 @@
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B33" s="3">
         <v>44</v>
       </c>
       <c r="C33" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="D33" t="s">
+        <v>124</v>
+      </c>
+      <c r="E33" s="4" t="s">
         <v>46</v>
-      </c>
-      <c r="D33" t="s">
-        <v>129</v>
-      </c>
-      <c r="E33" s="4" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B34" s="3">
         <v>38</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D34" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B35" s="3">
         <v>12</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D35" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="E35" s="2"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B36" s="3">
         <v>8</v>
       </c>
       <c r="C36" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="D36" t="s">
+        <v>126</v>
+      </c>
+      <c r="E36" s="2"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A37" s="7" t="s">
         <v>50</v>
-      </c>
-      <c r="D36" t="s">
-        <v>131</v>
-      </c>
-      <c r="E36" s="2"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="5" t="s">
-        <v>51</v>
       </c>
       <c r="B37" s="6"/>
       <c r="C37" s="6"/>
@@ -1405,39 +1409,39 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B38" s="3">
         <v>48</v>
       </c>
       <c r="C38" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="D38" t="s">
+        <v>127</v>
+      </c>
+      <c r="E38" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="D38" t="s">
-        <v>132</v>
-      </c>
-      <c r="E38" s="4" t="s">
-        <v>53</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B39" s="3">
         <v>4</v>
       </c>
       <c r="C39" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="D39" t="s">
+        <v>128</v>
+      </c>
+      <c r="E39" s="2"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A40" s="7" t="s">
         <v>54</v>
-      </c>
-      <c r="D39" t="s">
-        <v>133</v>
-      </c>
-      <c r="E39" s="2"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="5" t="s">
-        <v>55</v>
       </c>
       <c r="B40" s="6"/>
       <c r="C40" s="6"/>
@@ -1446,39 +1450,39 @@
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B41" s="3">
         <v>6</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D41" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="E41" s="2"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" s="2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B42" s="3">
         <v>2</v>
       </c>
       <c r="C42" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D42" t="s">
+        <v>137</v>
+      </c>
+      <c r="E42" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" s="7" t="s">
         <v>57</v>
-      </c>
-      <c r="D42" t="s">
-        <v>142</v>
-      </c>
-      <c r="E42" s="4" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="5" t="s">
-        <v>58</v>
       </c>
       <c r="B43" s="6"/>
       <c r="C43" s="6"/>
@@ -1487,37 +1491,37 @@
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B44" s="3">
         <v>1</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D44" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="E44" s="2"/>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B45" s="3">
         <v>1</v>
       </c>
       <c r="C45" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D45" t="s">
+        <v>130</v>
+      </c>
+      <c r="E45" s="2"/>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A46" s="7" t="s">
         <v>60</v>
-      </c>
-      <c r="D45" t="s">
-        <v>135</v>
-      </c>
-      <c r="E45" s="2"/>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A46" s="5" t="s">
-        <v>61</v>
       </c>
       <c r="B46" s="6"/>
       <c r="C46" s="6"/>
@@ -1526,92 +1530,92 @@
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B47" s="3">
         <v>10</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D47" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B48" s="3">
         <v>8</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D48" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B49" s="3">
         <v>2</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D49" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B50" s="3">
         <v>2</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D50" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" s="2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B51" s="3">
         <v>1</v>
       </c>
       <c r="C51" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="D51" t="s">
+        <v>146</v>
+      </c>
+      <c r="E51" s="4" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="7" t="s">
         <v>67</v>
-      </c>
-      <c r="D51" t="s">
-        <v>151</v>
-      </c>
-      <c r="E51" s="4" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A52" s="5" t="s">
-        <v>68</v>
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="6"/>
@@ -1620,109 +1624,109 @@
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B53" s="3">
         <v>4</v>
       </c>
       <c r="C53" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="D53" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E53" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="D53" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="E53" s="4" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B54" s="3">
         <v>2</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D54" s="2" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B55" s="3">
         <v>2</v>
       </c>
       <c r="C55" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="D55" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E55" s="4" t="s">
         <v>72</v>
-      </c>
-      <c r="D55" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="E55" s="4" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B56" s="3">
         <v>2</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D56" s="2" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B57" s="3">
         <v>1</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D57" s="2" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" s="2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B58" s="3">
         <v>1</v>
       </c>
       <c r="C58" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="D58" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="E58" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="7" t="s">
         <v>76</v>
-      </c>
-      <c r="D58" s="2" t="s">
-        <v>136</v>
-      </c>
-      <c r="E58" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A59" s="5" t="s">
-        <v>77</v>
       </c>
       <c r="B59" s="6"/>
       <c r="C59" s="6"/>
@@ -1731,24 +1735,24 @@
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B60" s="3">
         <v>2</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D60" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="E60" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="7" t="s">
         <v>78</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A61" s="5" t="s">
-        <v>79</v>
       </c>
       <c r="B61" s="6"/>
       <c r="C61" s="6"/>
@@ -1757,67 +1761,67 @@
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B62" s="3">
         <v>2</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>80</v>
+        <v>155</v>
       </c>
       <c r="D62" s="2"/>
       <c r="E62" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B63" s="3">
         <v>2</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D63" s="2"/>
       <c r="E63" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B64" s="3">
         <v>1</v>
       </c>
       <c r="C64" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="D64" s="2"/>
       <c r="E64" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B65" s="3">
         <v>1</v>
       </c>
       <c r="C65" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="D65" s="2"/>
       <c r="E65" s="2" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A66" s="5" t="s">
-        <v>84</v>
+      <c r="A66" s="7" t="s">
+        <v>82</v>
       </c>
       <c r="B66" s="6"/>
       <c r="C66" s="6"/>
@@ -1826,20 +1830,20 @@
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B67" s="3">
         <v>4</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="D67" s="2"/>
       <c r="E67" s="2"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A68" s="5" t="s">
-        <v>86</v>
+      <c r="A68" s="7" t="s">
+        <v>84</v>
       </c>
       <c r="B68" s="6"/>
       <c r="C68" s="6"/>
@@ -1848,48 +1852,48 @@
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B69" s="3">
         <v>2</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D69" s="2"/>
       <c r="E69" s="2"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B70" s="3">
         <v>1</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>88</v>
+        <v>152</v>
       </c>
       <c r="D70" s="2"/>
       <c r="E70" s="4" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="2" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B71" s="3">
         <v>1</v>
       </c>
       <c r="C71" s="2" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="D71" s="2"/>
       <c r="E71" s="2"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A72" s="5" t="s">
-        <v>91</v>
+      <c r="A72" s="7" t="s">
+        <v>88</v>
       </c>
       <c r="B72" s="6"/>
       <c r="C72" s="6"/>
@@ -1898,291 +1902,298 @@
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B73" s="3">
         <v>4</v>
       </c>
       <c r="C73" s="2" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="D73" s="2"/>
       <c r="E73" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B74" s="3">
         <v>4</v>
       </c>
       <c r="C74" s="2" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D74" s="2"/>
       <c r="E74" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B75" s="3">
         <v>4</v>
       </c>
       <c r="C75" s="2" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="D75" s="2"/>
       <c r="E75" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B76" s="3">
         <v>2</v>
       </c>
       <c r="C76" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D76" s="2"/>
       <c r="E76" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B77" s="3">
         <v>2</v>
       </c>
       <c r="C77" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D77" s="2"/>
       <c r="E77" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B78" s="3">
         <v>2</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D78" s="2"/>
       <c r="E78" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B79" s="3">
         <v>2</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D79" s="2"/>
       <c r="E79" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B80" s="3">
         <v>1</v>
       </c>
       <c r="C80" s="2" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="D80" s="2"/>
       <c r="E80" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B81" s="3">
         <v>1</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D81" s="2"/>
       <c r="E81" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B82" s="3">
         <v>1</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="D82" s="2"/>
       <c r="E82" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B83" s="3">
         <v>1</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D83" s="2"/>
       <c r="E83" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B84" s="3">
         <v>1</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>103</v>
+        <v>153</v>
       </c>
       <c r="D84" s="2"/>
       <c r="E84" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B85" s="3">
         <v>1</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>104</v>
+        <v>154</v>
       </c>
       <c r="D85" s="2"/>
       <c r="E85" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B86" s="3">
         <v>1</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="D86" s="2"/>
       <c r="E86" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B87" s="3">
         <v>1</v>
       </c>
       <c r="C87" s="2" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="D87" s="2"/>
       <c r="E87" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B88" s="3">
         <v>1</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="D88" s="2"/>
       <c r="E88" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B89" s="3">
         <v>1</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D89" s="2"/>
       <c r="E89" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B90" s="3">
         <v>1</v>
       </c>
       <c r="C90" s="2" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="D90" s="2"/>
       <c r="E90" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" s="2" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B91" s="3">
         <v>1</v>
       </c>
       <c r="C91" s="2" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="D91" s="2"/>
       <c r="E91" s="4" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="20">
+    <mergeCell ref="A72:E72"/>
+    <mergeCell ref="A52:E52"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A68:E68"/>
+    <mergeCell ref="A40:E40"/>
+    <mergeCell ref="A59:E59"/>
+    <mergeCell ref="A66:E66"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A61:E61"/>
     <mergeCell ref="A25:E25"/>
@@ -2195,14 +2206,7 @@
     <mergeCell ref="A5:E5"/>
     <mergeCell ref="A23:E23"/>
     <mergeCell ref="A20:E20"/>
-    <mergeCell ref="A72:E72"/>
-    <mergeCell ref="A52:E52"/>
-    <mergeCell ref="A43:E43"/>
-    <mergeCell ref="A68:E68"/>
-    <mergeCell ref="A40:E40"/>
     <mergeCell ref="A30:E30"/>
-    <mergeCell ref="A59:E59"/>
-    <mergeCell ref="A66:E66"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Printed: XY joint M4 holes moved 0.99 mm to match the stock SV08 toolhead extrusion
Holes now 5 mm and 25 mm from the extrusion ends, like the stock holes; outlines grown 0.54 mm,
end walls 2.0 mm (accepted). Main, XY joint assemblies, STL previews, renders and BOM notes updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Printed Version/SV08_P6_Printed_BOM_from_STEP.xlsx
+++ b/Printed Version/SV08_P6_Printed_BOM_from_STEP.xlsx
@@ -1314,7 +1314,7 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
-          <t>6mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions.</t>
+          <t>6mm OD is more common and acceptable. Purchase preferred. Printed as alternative with same dimensions. Optional: use a 6mm OD (or smaller) spacer for the one nearest each end of the Gantry X extrusion (2 total) and the stock 345mm extrusion fits without cutting.</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,11 @@
         </is>
       </c>
       <c r="D70" s="2" t="n"/>
-      <c r="E70" s="2" t="n"/>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Stock extrusion works: the front and back motor-mount bolt holes line up with its existing holes.</t>
+        </is>
+      </c>
     </row>
     <row r="71" s="6">
       <c r="A71" s="2" t="inlineStr">
@@ -1795,7 +1799,7 @@
       <c r="D71" s="2" t="n"/>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>Shortened from 345mm: all tensioning now happens at the front motor mounts.</t>
+          <t>Shortened from 345mm: all tensioning now happens at the front motor mounts. The back motor-mount bolt holes line up with the stock extrusion's existing holes. To use the stock 345mm extrusion without cutting it, fit a 6mm OD (or smaller) M3 x 20mm spacer in the spot nearest each end of this extrusion (one per back corner) instead of an 8mm one.</t>
         </is>
       </c>
     </row>
@@ -1814,7 +1818,11 @@
         </is>
       </c>
       <c r="D72" s="2" t="n"/>
-      <c r="E72" s="2" t="n"/>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Stock extrusion works: the XY joint bolt holes line up with its existing holes (5mm and 25mm from each end).</t>
+        </is>
+      </c>
     </row>
     <row r="73" s="6">
       <c r="A73" s="7" t="inlineStr">

</xml_diff>

<commit_message>
Printed: Chicago bolt live idler shafts; stock parts models; stock extrusion notes
Printed fronts and XY joints now use 304 stainless Chicago bolt bases (30/40 mm, 5 mm barrel)
with M4x8 ultra-thin flat heads: full-width, clamped bearings, 0.4 mm under the front motors
(front plate pocket floors 4.4 -> 4.6). Printed BOM: Live Idler Shafts section replaces the
threaded spacers and M3 ultra-thin heads (kept as alternatives). New Shared Components/Stock
Parts: Chicago bolt parts and the stock SV08 toolhead / gantry X / gantry Y extrusions.
BOMs (all versions): trim the 345 mm gantry X 1.5 mm per end. New 3MF, STL previews, renders,
README notes.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Printed Version/SV08_P6_Printed_BOM_from_STEP.xlsx
+++ b/Printed Version/SV08_P6_Printed_BOM_from_STEP.xlsx
@@ -653,21 +653,21 @@
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>M3 x 10mm Ultra Thin Flat Head (.8-1mm)</t>
+          <t>M4x8 Ultra Thin Flat Head</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0H61WCTBX</t>
+          <t>https://amazon.com/dp/B0H61X7SWB</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Ultra-thin head (.8-1mm). 2 per front motor assembly and 2 per XY joint. Use threadlocker: blue (medium, removable) recommended; red (high strength) only for a permanent build, since removing it takes heat that can damage bearings and printed parts.</t>
+          <t>Screw end of each Chicago bolt live idler shaft (1 per front motor assembly and 1 per XY joint). 1.2mm head, thin enough to clear the front motors. Use threadlocker: blue (medium, removable) recommended; red (high strength) only for a permanent build, since removing it takes heat that can damage bearings and printed parts.</t>
         </is>
       </c>
     </row>
@@ -872,14 +872,14 @@
     <row r="22" s="6">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Fasteners - Threaded Rods</t>
+          <t>Live Idler Shafts</t>
         </is>
       </c>
     </row>
     <row r="23" s="6">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Threaded Rods</t>
+          <t>Live Idler Shafts</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
@@ -887,24 +887,24 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>M3 Internally Threaded Spacer (5mm OD | 35mm Tall)</t>
+          <t>M5x40 Chicago Bolt Base</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0D3HWQ2GF</t>
+          <t>https://amazon.com/dp/B0FLJNY14R</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Replaces the M5 x 40mm dowel in the XY Joints (1 per joint). Clamped between the plates by 2x M3 x 10mm Ultra Thin Flat Head per joint. It reaches 1.5 mm into each bearing. A 40 mm spacer would run through both bearings for their full width, but the 35 mm is kept so the same part fits every version of the build. FIT NOTE: the spacers measure about 5.05 mm across (anodised aluminium), a little too big for the 4.992-5.000 mm bore of a 695 bearing, so sand the whole length of each spacer down to fit, not just the ends: the toothed pulley or idler has to slide along the shaft to reach its place between the bearings, and sanding only the last 5 mm of each end isn't enough. This is common practice in the 3D printing community, and it's confirmed working on the v2 test build. Spin the spacer in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go (aim for about 4.990-4.995 mm), and stop when it presses into a bearing with firm thumb pressure and the pulley slides over it. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 40 mm long, works in place of the spacer and its two flat-head screws. At 40 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. Test-fit each dowel in a bearing before assembly and sand or grind it to size the same way if it's tight. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
+          <t>Live idler shaft in the XY joints (1 per joint). 304 stainless Chicago screw: the 5mm x 40mm barrel runs the full width of both bearings, its head on one bearing and an M4x8 Ultra Thin Flat Head on the other, so the bearings are clamped and the idler can't float. Pack of 20. The M4x4 screws in the pack aren't used: their 2mm heads don't clear the front motors, so the ultra-thin heads are used everywhere. ALTERNATIVES (not as good): an M3 internally threaded spacer, 5mm OD x 35mm (amazon.com/dp/B0D3HWQ2GF), clamped by 2x M3 x 10mm ultra-thin flat heads (amazon.com/dp/B0H61WCTBX). The anodised spacers measure about 5.05mm, so sand the whole length in a drill (400-600 grit) until it presses into a bearing with firm thumb pressure and the pulley slides over it. Or a 5mm h6/h7 slip-fit dowel / ground shaft, 40mm long: it fits, but it's held only by the pulley set screws, so the idler can float up and down under belt tension, which causes vibration.</t>
         </is>
       </c>
     </row>
     <row r="24" s="6">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>Threaded Rods</t>
+          <t>Live Idler Shafts</t>
         </is>
       </c>
       <c r="B24" s="3" t="n">
@@ -912,17 +912,17 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>M3 Internally Threaded Spacer (5mm OD | 25mm Tall)</t>
+          <t>M5x30 Chicago Bolt Base</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://amazon.com/dp/B0D3HVVJPN</t>
+          <t>https://amazon.com/dp/B0FLJQP39V</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Replaces the M5 x 30mm dowel in the front motor assemblies (1 per side). Held by 2x M3 x 10mm Ultra Thin Flat Head. FIT NOTE: the spacers measure about 5.05 mm across (anodised aluminium), a little too big for the 4.992-5.000 mm bore of a 695 bearing, so sand the whole length of each spacer down to fit, not just the ends: the toothed pulley or idler has to slide along the shaft to reach its place between the bearings, and sanding only the last 5 mm of each end isn't enough. This is common practice in the 3D printing community, and it's confirmed working on the v2 test build. Spin the spacer in a drill against 400-600 grit, or roll it under a flat block on sandpaper laid on the bench. Measure in two directions as you go (aim for about 4.990-4.995 mm), and stop when it presses into a bearing with firm thumb pressure and the pulley slides over it. Don't force an oversize spacer in; that loads the bearing balls. ALTERNATIVE: a 5 mm dowel pin, 30 mm long, works in place of the spacer and its two flat-head screws. At 30 mm it runs the full width of both bearings, flush with their outer faces. Get h6/h7 (slip-fit) dowels or a cut length of 5 mm ground linear shaft (h6/g6): standard m6 press-fit dowels are 5.004-5.012 mm and will jam in the bearing just like the oversize spacers. Test-fit each dowel in a bearing before assembly and sand or grind it to size the same way if it's tight. The pulley's set screws hold the dowel in place, and the pulley sits between the two bearings.</t>
+          <t>Live idler shaft in the front motor assemblies (1 per side). 304 stainless Chicago screw: the 5mm x 30mm barrel runs the full width of both bearings, head at the bottom and an M4x8 Ultra Thin Flat Head at the top, 0.4mm under the motor. Pack of 20; the M4x4 screws in the pack aren't used (their 2mm heads don't clear the motor). ALTERNATIVES (not as good): an M3 internally threaded spacer, 5mm OD x 25mm (amazon.com/dp/B0D3HVVJPN), clamped by 2x M3 x 10mm ultra-thin flat heads (amazon.com/dp/B0H61WCTBX). The anodised spacers measure about 5.05mm, so sand the whole length in a drill (400-600 grit) until it presses into a bearing with firm thumb pressure and the pulley slides over it. Or a 5mm h6/h7 slip-fit dowel / ground shaft, 30mm long: it fits, but it's held only by the pulley set screws, so the idler can float up and down under belt tension, which causes vibration.</t>
         </is>
       </c>
     </row>
@@ -1799,7 +1799,7 @@
       <c r="D71" s="2" t="n"/>
       <c r="E71" s="4" t="inlineStr">
         <is>
-          <t>Shortened from 345mm: all tensioning now happens at the front motor mounts. The back motor-mount bolt holes line up with the stock extrusion's existing holes. To use the stock 345mm extrusion without cutting it, fit a 6mm OD (or smaller) M3 x 20mm spacer in the spot nearest each end of this extrusion (one per back corner) instead of an 8mm one.</t>
+          <t>Shortened from 345mm: all tensioning now happens at the front motor mounts. The back motor-mount bolt holes line up with the stock extrusion's existing holes. To use the stock 345mm extrusion without cutting it, fit a 6mm OD (or smaller) M3 x 20mm spacer in the spot nearest each end of this extrusion (one per back corner) instead of an 8mm one. If you cut a 345mm extrusion down to 342mm, take 1.5mm off each end: the stock holes are 5mm and 23mm from each end, so an even trim keeps both ends lined up with the back motor-mount holes.</t>
         </is>
       </c>
     </row>

</xml_diff>